<commit_message>
introduced feed in e from grid
</commit_message>
<xml_diff>
--- a/Dataset/MappingConDatiArticolo.xlsx
+++ b/Dataset/MappingConDatiArticolo.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristian/PycharmProjects/EnergyOptimization/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE4FD0F4-EABB-4445-909C-441761176180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED62B2C-985B-A648-AA31-4DF10332633C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{ADBE4949-0076-D64E-ACAC-FDF7396AF500}"/>
+    <workbookView xWindow="4400" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{ADBE4949-0076-D64E-ACAC-FDF7396AF500}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
   <si>
     <t> Discharge(Wh)</t>
   </si>
@@ -101,12 +101,6 @@
     <t>vP_PV</t>
   </si>
   <si>
-    <t>vP_S_c</t>
-  </si>
-  <si>
-    <t>vP_S_d</t>
-  </si>
-  <si>
     <t>Pgtd = Egtd / 60 (se &lt; 0, 60 perché è un minuto)</t>
   </si>
   <si>
@@ -141,6 +135,9 @@
   </si>
   <si>
     <t>Output</t>
+  </si>
+  <si>
+    <t>vP_S</t>
   </si>
 </sst>
 </file>
@@ -560,12 +557,12 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -591,10 +588,10 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="F3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
         <v>14</v>
@@ -602,25 +599,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>7</v>
@@ -649,13 +646,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>13</v>
@@ -664,24 +661,24 @@
         <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
bug fixing asp program
</commit_message>
<xml_diff>
--- a/Dataset/MappingConDatiArticolo.xlsx
+++ b/Dataset/MappingConDatiArticolo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristian/PycharmProjects/EnergyOptimization/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED62B2C-985B-A648-AA31-4DF10332633C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DDA050-9F57-A54E-AB2B-61D01D3D582A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4400" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{ADBE4949-0076-D64E-ACAC-FDF7396AF500}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{ADBE4949-0076-D64E-ACAC-FDF7396AF500}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t> Discharge(Wh)</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>vP_S</t>
+  </si>
+  <si>
+    <t>vP_G</t>
   </si>
 </sst>
 </file>
@@ -686,6 +689,12 @@
       <c r="E8" t="s">
         <v>19</v>
       </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>